<commit_message>
update to Kafka links .xcel
</commit_message>
<xml_diff>
--- a/SEVEN_Kakfa_Links.xlsx
+++ b/SEVEN_Kakfa_Links.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\A233C1F\Documents\Docs&amp;Misc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3664EEC-650E-412B-A9F5-AAC03C764DC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AB9DCB9-5910-4813-A7C7-9A3AE88246CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="1050" windowWidth="29040" windowHeight="15720" xr2:uid="{9D751822-9D83-4D60-B2B6-9E7CF2D78AD8}"/>
   </bookViews>
   <sheets>
     <sheet name="Links" sheetId="1" r:id="rId1"/>
     <sheet name="Kafka Self Service" sheetId="2" r:id="rId2"/>
+    <sheet name="RTP" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="38">
   <si>
     <t>https://rewe.atlassian.net/wiki/spaces/TITISEVEN/pages/1134952479/System+overview+Kafka+Clusters+managed+by+Team+SEVEN</t>
   </si>
@@ -90,9 +91,6 @@
     <t>Kafka Self-Service</t>
   </si>
   <si>
-    <t>https://code.dev.rewe.cloud/ip/caas/kafka-self-service</t>
-  </si>
-  <si>
     <t>https://rewe.atlassian.net/wiki/spaces/GBOS/pages/1260465890/Use+REWE+Kafka+topic+naming+convention</t>
   </si>
   <si>
@@ -223,6 +221,22 @@
   </si>
   <si>
     <t>https://code.dev.rewe.cloud/ip/caas/kafka-self-service-pipeline</t>
+  </si>
+  <si>
+    <t>Ulbrich, Robert: https://gitlab.cicd.rewe.cloud/rewe-tech-platform/prod633/applica... | Provisioning of Mirrormakers for RTP | Microsoft Teams</t>
+  </si>
+  <si>
+    <t>https://gitlab.cicd.rewe.cloud/rewe-tech-platform/prod633/applications/kafka-test/kafka-test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RTP </t>
+  </si>
+  <si>
+    <t>Engineer on duty</t>
+  </si>
+  <si>
+    <t>https://code.dev.rewe.cloud/ip/caas/kafka-self-service
+https://code.dev.rewe.cloud/ip/caas/kafka-self-service/-/merge_requests</t>
   </si>
 </sst>
 </file>
@@ -291,7 +305,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -315,6 +329,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -668,23 +691,23 @@
   <cols>
     <col min="1" max="1" width="19.54296875" customWidth="1"/>
     <col min="2" max="2" width="120" customWidth="1"/>
-    <col min="3" max="3" width="13.26953125" customWidth="1"/>
+    <col min="3" max="3" width="14.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
         <v>16</v>
       </c>
-      <c r="B3" t="s">
-        <v>17</v>
-      </c>
       <c r="C3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="58" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>0</v>
@@ -700,10 +723,10 @@
     </row>
     <row r="6" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="29" x14ac:dyDescent="0.35">
@@ -730,55 +753,58 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10" s="5" t="s">
+    <row r="10" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A10" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="3" t="s">
-        <v>10</v>
+      <c r="B10" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -787,17 +813,18 @@
     <hyperlink ref="B7" r:id="rId2" xr:uid="{73492074-DA97-44C4-90AF-C79CF5DBA21C}"/>
     <hyperlink ref="B8" r:id="rId3" xr:uid="{EB59DAC2-E5D5-4D34-943B-42B2CB5423FF}"/>
     <hyperlink ref="B9" r:id="rId4" xr:uid="{4E33CBEF-9533-48D2-BC67-45717AA3FBEB}"/>
-    <hyperlink ref="B10" r:id="rId5" xr:uid="{05DBEA20-3695-490C-93E6-102AAED9E6DE}"/>
+    <hyperlink ref="B10" r:id="rId5" display="https://code.dev.rewe.cloud/ip/caas/kafka-self-service" xr:uid="{05DBEA20-3695-490C-93E6-102AAED9E6DE}"/>
     <hyperlink ref="B11" r:id="rId6" xr:uid="{A82AE5B1-B074-4F20-A1EE-F4A97F50477A}"/>
     <hyperlink ref="B12" r:id="rId7" xr:uid="{4233B4E2-FA5D-4231-82C5-0DEBEE98C968}"/>
     <hyperlink ref="B13" r:id="rId8" xr:uid="{F04C5879-D231-445B-930D-ECD231A12A54}"/>
     <hyperlink ref="B14" r:id="rId9" xr:uid="{5A6AE6C9-548A-4156-8643-080D848DAC3C}"/>
     <hyperlink ref="B6" r:id="rId10" xr:uid="{67284D87-5311-488E-912B-0A02FF85032A}"/>
+    <hyperlink ref="B5" r:id="rId11" xr:uid="{997FA379-5083-4A11-A6D1-809BA5407CED}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId11"/>
+  <pageSetup orientation="portrait" r:id="rId12"/>
   <tableParts count="1">
-    <tablePart r:id="rId12"/>
+    <tablePart r:id="rId13"/>
   </tableParts>
 </worksheet>
 </file>
@@ -813,31 +840,31 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>32</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -848,4 +875,33 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C234A6A-5C6C-4377-8976-D599C42620F0}">
+  <dimension ref="E3:E5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="3" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E4" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E5" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E4" r:id="rId1" display="https://teams.microsoft.com/l/message/19:meeting_NWM2NjU4MGItN2JhMy00NGJiLWEwOTItNmNhOTc5ZTUxMzY3@thread.v2/1772458060267?context=%7B%22contextType%22%3A%22chat%22%7D" xr:uid="{090EFF01-141B-4203-9C19-FEAA5A9787AA}"/>
+    <hyperlink ref="E5" r:id="rId2" xr:uid="{2FAFDE5F-C7BC-44D2-B43D-3A7B95C1978C}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Updates to MQ and Kafka notes
</commit_message>
<xml_diff>
--- a/SEVEN_Kakfa_Links.xlsx
+++ b/SEVEN_Kakfa_Links.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\A233C1F\Documents\Docs&amp;Misc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AB9DCB9-5910-4813-A7C7-9A3AE88246CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3B7F094-9F14-4C8F-BD17-A0FCC275DCA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="1050" windowWidth="29040" windowHeight="15720" xr2:uid="{9D751822-9D83-4D60-B2B6-9E7CF2D78AD8}"/>
+    <workbookView xWindow="-28920" yWindow="1050" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{9D751822-9D83-4D60-B2B6-9E7CF2D78AD8}"/>
   </bookViews>
   <sheets>
     <sheet name="Links" sheetId="1" r:id="rId1"/>
     <sheet name="Kafka Self Service" sheetId="2" r:id="rId2"/>
     <sheet name="RTP" sheetId="3" r:id="rId3"/>
+    <sheet name="Change control" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="41">
   <si>
     <t>https://rewe.atlassian.net/wiki/spaces/TITISEVEN/pages/1134952479/System+overview+Kafka+Clusters+managed+by+Team+SEVEN</t>
   </si>
@@ -237,6 +238,15 @@
   <si>
     <t>https://code.dev.rewe.cloud/ip/caas/kafka-self-service
 https://code.dev.rewe.cloud/ip/caas/kafka-self-service/-/merge_requests</t>
+  </si>
+  <si>
+    <t>https://servicedesk.eil.risnet.de/browse/CHANGE-3763</t>
+  </si>
+  <si>
+    <t>https://teams.microsoft.com/l/message/19:meeting_ODFhYWYxOWYtMjAwMC00MjgyLTliNjItOTZkNjU2Y2IzNmE2@thread.v2/1772627431981?context=%7B%22contextType%22%3A%22chat%22%7D</t>
+  </si>
+  <si>
+    <t>O&amp;M migration</t>
   </si>
 </sst>
 </file>
@@ -355,6 +365,55 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>344054</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>105623</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{54A321B2-EAC1-E41F-5B01-12E88BEE826D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="8268854" cy="6077798"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -904,4 +963,34 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CF4F27D-A951-431B-81D5-DDDFCFE35034}">
+  <dimension ref="O11:O13"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="11" spans="15:15" x14ac:dyDescent="0.35">
+      <c r="O11" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="15:15" x14ac:dyDescent="0.35">
+      <c r="O12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" spans="15:15" x14ac:dyDescent="0.35">
+      <c r="O13" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="O11" r:id="rId1" xr:uid="{4AB133D0-16BC-4751-927B-F13972E7426F}"/>
+    <hyperlink ref="O13" r:id="rId2" xr:uid="{0C18E59B-8920-4BF4-A56A-04786EB994F8}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
links updates abs new GO sample code added
</commit_message>
<xml_diff>
--- a/SEVEN_Kakfa_Links.xlsx
+++ b/SEVEN_Kakfa_Links.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\A233C1F\Documents\Docs&amp;Misc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3B7F094-9F14-4C8F-BD17-A0FCC275DCA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B55E587-603C-43A5-B19E-B423DD2349AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="1050" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{9D751822-9D83-4D60-B2B6-9E7CF2D78AD8}"/>
+    <workbookView xWindow="-21945" yWindow="5055" windowWidth="19515" windowHeight="11610" activeTab="1" xr2:uid="{9D751822-9D83-4D60-B2B6-9E7CF2D78AD8}"/>
   </bookViews>
   <sheets>
     <sheet name="Links" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="43">
   <si>
     <t>https://rewe.atlassian.net/wiki/spaces/TITISEVEN/pages/1134952479/System+overview+Kafka+Clusters+managed+by+Team+SEVEN</t>
   </si>
@@ -247,6 +247,12 @@
   </si>
   <si>
     <t>O&amp;M migration</t>
+  </si>
+  <si>
+    <t>https://it-insights-api.rewe.local/swagger-ui/index.html</t>
+  </si>
+  <si>
+    <t>IT insight API</t>
   </si>
 </sst>
 </file>
@@ -879,18 +885,19 @@
     <hyperlink ref="B14" r:id="rId9" xr:uid="{5A6AE6C9-548A-4156-8643-080D848DAC3C}"/>
     <hyperlink ref="B6" r:id="rId10" xr:uid="{67284D87-5311-488E-912B-0A02FF85032A}"/>
     <hyperlink ref="B5" r:id="rId11" xr:uid="{997FA379-5083-4A11-A6D1-809BA5407CED}"/>
+    <hyperlink ref="B15" r:id="rId12" xr:uid="{3F6F8243-51FF-46D2-9E1F-36AA9EE212C8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId12"/>
+  <pageSetup orientation="portrait" r:id="rId13"/>
   <tableParts count="1">
-    <tablePart r:id="rId13"/>
+    <tablePart r:id="rId14"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A03D07D-390D-4964-84B8-DA4DC0A69C33}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="62.08984375" customWidth="1"/>
@@ -926,11 +933,20 @@
         <v>32</v>
       </c>
     </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B3" r:id="rId1" xr:uid="{0C302664-FE7C-45B4-B81E-F297190B1C6D}"/>
     <hyperlink ref="B6" r:id="rId2" xr:uid="{6ECA404E-1699-4097-B9D5-BCF71406C79C}"/>
     <hyperlink ref="B7" r:id="rId3" xr:uid="{FD83F1CF-F75B-4B95-8D92-29CEF8DC3234}"/>
+    <hyperlink ref="B10" r:id="rId4" xr:uid="{9EE5D787-F140-4202-BA2B-C8A2446AD6E4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
links updates and new GO sample code added
</commit_message>
<xml_diff>
--- a/SEVEN_Kakfa_Links.xlsx
+++ b/SEVEN_Kakfa_Links.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\A233C1F\Documents\Docs&amp;Misc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3B7F094-9F14-4C8F-BD17-A0FCC275DCA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B55E587-603C-43A5-B19E-B423DD2349AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="1050" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{9D751822-9D83-4D60-B2B6-9E7CF2D78AD8}"/>
+    <workbookView xWindow="-21945" yWindow="5055" windowWidth="19515" windowHeight="11610" activeTab="1" xr2:uid="{9D751822-9D83-4D60-B2B6-9E7CF2D78AD8}"/>
   </bookViews>
   <sheets>
     <sheet name="Links" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="43">
   <si>
     <t>https://rewe.atlassian.net/wiki/spaces/TITISEVEN/pages/1134952479/System+overview+Kafka+Clusters+managed+by+Team+SEVEN</t>
   </si>
@@ -247,6 +247,12 @@
   </si>
   <si>
     <t>O&amp;M migration</t>
+  </si>
+  <si>
+    <t>https://it-insights-api.rewe.local/swagger-ui/index.html</t>
+  </si>
+  <si>
+    <t>IT insight API</t>
   </si>
 </sst>
 </file>
@@ -879,18 +885,19 @@
     <hyperlink ref="B14" r:id="rId9" xr:uid="{5A6AE6C9-548A-4156-8643-080D848DAC3C}"/>
     <hyperlink ref="B6" r:id="rId10" xr:uid="{67284D87-5311-488E-912B-0A02FF85032A}"/>
     <hyperlink ref="B5" r:id="rId11" xr:uid="{997FA379-5083-4A11-A6D1-809BA5407CED}"/>
+    <hyperlink ref="B15" r:id="rId12" xr:uid="{3F6F8243-51FF-46D2-9E1F-36AA9EE212C8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId12"/>
+  <pageSetup orientation="portrait" r:id="rId13"/>
   <tableParts count="1">
-    <tablePart r:id="rId13"/>
+    <tablePart r:id="rId14"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A03D07D-390D-4964-84B8-DA4DC0A69C33}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="62.08984375" customWidth="1"/>
@@ -926,11 +933,20 @@
         <v>32</v>
       </c>
     </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B3" r:id="rId1" xr:uid="{0C302664-FE7C-45B4-B81E-F297190B1C6D}"/>
     <hyperlink ref="B6" r:id="rId2" xr:uid="{6ECA404E-1699-4097-B9D5-BCF71406C79C}"/>
     <hyperlink ref="B7" r:id="rId3" xr:uid="{FD83F1CF-F75B-4B95-8D92-29CEF8DC3234}"/>
+    <hyperlink ref="B10" r:id="rId4" xr:uid="{9EE5D787-F140-4202-BA2B-C8A2446AD6E4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
updates to kafka links
</commit_message>
<xml_diff>
--- a/SEVEN_Kakfa_Links.xlsx
+++ b/SEVEN_Kakfa_Links.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\A233C1F\Documents\Docs&amp;Misc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B55E587-603C-43A5-B19E-B423DD2349AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C20D58F5-AA74-4385-84BC-BA2B51E978C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21945" yWindow="5055" windowWidth="19515" windowHeight="11610" activeTab="1" xr2:uid="{9D751822-9D83-4D60-B2B6-9E7CF2D78AD8}"/>
+    <workbookView xWindow="-22860" yWindow="4515" windowWidth="19515" windowHeight="11610" activeTab="1" xr2:uid="{9D751822-9D83-4D60-B2B6-9E7CF2D78AD8}"/>
   </bookViews>
   <sheets>
     <sheet name="Links" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="44">
   <si>
     <t>https://rewe.atlassian.net/wiki/spaces/TITISEVEN/pages/1134952479/System+overview+Kafka+Clusters+managed+by+Team+SEVEN</t>
   </si>
@@ -253,6 +253,10 @@
   </si>
   <si>
     <t>IT insight API</t>
+  </si>
+  <si>
+    <t>change .gitlab-ci.yml updating the version
+change README.md</t>
   </si>
 </sst>
 </file>
@@ -321,7 +325,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -354,6 +358,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -897,19 +904,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A03D07D-390D-4964-84B8-DA4DC0A69C33}">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="62.08984375" customWidth="1"/>
     <col min="2" max="2" width="73.54296875" customWidth="1"/>
+    <col min="3" max="3" width="23.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>28</v>
       </c>
@@ -917,15 +925,18 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
         <v>30</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C6" s="13" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>31</v>
       </c>
@@ -933,7 +944,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>42</v>
       </c>

</xml_diff>